<commit_message>
State the planning policies: safety stock, backorders, workers
- Beginning backorders are now given data with their own Excel name
  (BeginBackorders, 0 by default, instructor-configurable); the answer
  key, checker and hints start January from it.
- New "Planning policies" section on the Scenario and Start Here sheets
  and step 1 of the app (also on each plan step): what the safety-stock
  policy means for the chase, level and hybrid plans; how backorders
  carry forward and are charged; and the workforce rule.
- New worker_policy option: whole workers (round up, idle capacity is
  paid; default) or partial (fractional worker-equivalents). Answer key,
  checker, feasibility and hints follow it.
- Excel-calculated fixture with every policy switched; 92 tests pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/key_seed7.xlsx
+++ b/tests/fixtures/key_seed7.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cms89\AppData\Roaming\Claude\scratch-workspaces\a72c5ced-5896-445f-ba4c-143e77ffe85d\78e220c2-1d03-4db7-9c30-facaa620e845\scratch-2026-10-19-6e9fe4\v3\tests\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{30F7932B-A196-4AA7-B581-A1A4178E9808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{46AE3A6B-566C-4D34-A52A-32A4171435B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -23,23 +23,24 @@
     <sheet name="_meta" sheetId="8" state="veryHidden" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="BackorderCost">Scenario!$F$18</definedName>
+    <definedName name="BackorderCost">Scenario!$F$19</definedName>
+    <definedName name="BeginBackorders">Scenario!$F$7</definedName>
     <definedName name="BeginInv">Scenario!$F$6</definedName>
-    <definedName name="BottlesPerHour">Scenario!$F$11</definedName>
-    <definedName name="DaysPerMonth">Scenario!$F$13</definedName>
-    <definedName name="EndTarget">Scenario!$F$8</definedName>
-    <definedName name="HireCost">Scenario!$F$15</definedName>
-    <definedName name="HoldCost">Scenario!$F$17</definedName>
-    <definedName name="HoursPerDay">Scenario!$F$12</definedName>
-    <definedName name="LaborCost">Scenario!$F$14</definedName>
-    <definedName name="LayoffCost">Scenario!$F$16</definedName>
-    <definedName name="MaxInventory">Scenario!$F$9</definedName>
-    <definedName name="OTCost">Scenario!$F$20</definedName>
-    <definedName name="OTLimitPct">Scenario!$F$19</definedName>
-    <definedName name="SafetyStock">Scenario!$F$7</definedName>
-    <definedName name="StartWorkers">Scenario!$F$10</definedName>
-    <definedName name="SubCapacity">Scenario!$F$22</definedName>
-    <definedName name="SubCost">Scenario!$F$21</definedName>
+    <definedName name="BottlesPerHour">Scenario!$F$12</definedName>
+    <definedName name="DaysPerMonth">Scenario!$F$14</definedName>
+    <definedName name="EndTarget">Scenario!$F$9</definedName>
+    <definedName name="HireCost">Scenario!$F$16</definedName>
+    <definedName name="HoldCost">Scenario!$F$18</definedName>
+    <definedName name="HoursPerDay">Scenario!$F$13</definedName>
+    <definedName name="LaborCost">Scenario!$F$15</definedName>
+    <definedName name="LayoffCost">Scenario!$F$17</definedName>
+    <definedName name="MaxInventory">Scenario!$F$10</definedName>
+    <definedName name="OTCost">Scenario!$F$21</definedName>
+    <definedName name="OTLimitPct">Scenario!$F$20</definedName>
+    <definedName name="SafetyStock">Scenario!$F$8</definedName>
+    <definedName name="StartWorkers">Scenario!$F$11</definedName>
+    <definedName name="SubCapacity">Scenario!$F$23</definedName>
+    <definedName name="SubCost">Scenario!$F$22</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -134,7 +135,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="286">
   <si>
     <t>Aggregate Anxiety: Aggregate Planning in Excel</t>
   </si>
@@ -208,10 +209,64 @@
     <t>Yearly totals row (row 14)</t>
   </si>
   <si>
-    <t>Your company's policy</t>
-  </si>
-  <si>
-    <t>Your company carries no safety stock: the chase plan uses up the beginning inventory in January and then ends each month with 0 bottles; the level plan aims to end December at 0.</t>
+    <t>Your company's planning policies (every plan must follow them)</t>
+  </si>
+  <si>
+    <t>Safety stock: NONE</t>
+  </si>
+  <si>
+    <t>• Your company does NOT keep safety stock, so EndTarget = 0. The SafetyStock figure on the Scenario sheet is not used by your plans.</t>
+  </si>
+  <si>
+    <t>• Chase plan: use up the beginning inventory, then aim to end every month with 0 bottles on the shelf.</t>
+  </si>
+  <si>
+    <t>• Level plan: one steady rate, chosen so that December ends with 0 bottles.</t>
+  </si>
+  <si>
+    <t>• Hybrid plan: December may end with any stock of 0 or more.</t>
+  </si>
+  <si>
+    <t>• Beginning inventory (BeginInv = 2,400) is simply the stock on the shelf on January 1 — use it up; don't keep it as a reserve.</t>
+  </si>
+  <si>
+    <t>Backorders: unfilled orders carry forward</t>
+  </si>
+  <si>
+    <t>• An order you can't fill is not lost: it becomes a backorder and is still owed next month.</t>
+  </si>
+  <si>
+    <t>• You start the year owing BeginBackorders = 0 bottles of orders.</t>
+  </si>
+  <si>
+    <t>• When stock is available, old orders are shipped first, then this month's demand.</t>
+  </si>
+  <si>
+    <t>• Every bottle still on backorder at the end of a month costs BackorderCost for that month.</t>
+  </si>
+  <si>
+    <t>• Stock is never negative: a shortfall is recorded as backorders, not as negative inventory.</t>
+  </si>
+  <si>
+    <t>• Hybrid plan: no more than 0 bottles may still be on backorder at the end of December, and at least 95% of demand must ship in the month it is ordered.</t>
+  </si>
+  <si>
+    <t>Workforce: whole workers only</t>
+  </si>
+  <si>
+    <t>• You employ whole people — there are no fractions of a worker.</t>
+  </si>
+  <si>
+    <t>• If a month's production needs, say, 10.2 workers' worth of capacity, you must employ 11. The extra capacity sits idle, but those workers are still paid.</t>
+  </si>
+  <si>
+    <t>• Workers are paid LaborCost for every month they are employed, busy or not.</t>
+  </si>
+  <si>
+    <t>• You start the year with StartWorkers = 8 workers. Hiring and layoffs are counted against the previous month's workforce (January against StartWorkers): each hire costs HireCost, each layoff LayoffCost.</t>
+  </si>
+  <si>
+    <t>• One worker's monthly capacity comes from their output per hour, paid hours per day and working days per month (Scenario sheet).</t>
   </si>
   <si>
     <t>Questions every plan must answer, for each month</t>
@@ -352,22 +407,31 @@
     <t>February</t>
   </si>
   <si>
-    <t>Safety-stock quantity</t>
+    <t>Customer orders still unfilled before January</t>
+  </si>
+  <si>
+    <t>BeginBackorders</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>Safety-stock quantity (see Planning policies below)</t>
   </si>
   <si>
     <t>SafetyStock</t>
   </si>
   <si>
-    <t>March</t>
-  </si>
-  <si>
-    <t>Inventory each chase month aims to end with (and the level plan's December target)</t>
+    <t>April</t>
+  </si>
+  <si>
+    <t>Ending-inventory target your policy sets (see below)</t>
   </si>
   <si>
     <t>EndTarget</t>
   </si>
   <si>
-    <t>April</t>
+    <t>May</t>
   </si>
   <si>
     <t>Storage capacity (most bottles you can hold)</t>
@@ -376,7 +440,7 @@
     <t>MaxInventory</t>
   </si>
   <si>
-    <t>May</t>
+    <t>June</t>
   </si>
   <si>
     <t>Workers employed before January</t>
@@ -388,7 +452,7 @@
     <t>workers</t>
   </si>
   <si>
-    <t>June</t>
+    <t>July</t>
   </si>
   <si>
     <t>Output of one worker per hour</t>
@@ -400,7 +464,7 @@
     <t>bottles/hour</t>
   </si>
   <si>
-    <t>July</t>
+    <t>August</t>
   </si>
   <si>
     <t>Paid hours per worker per day</t>
@@ -412,7 +476,7 @@
     <t>hours/day</t>
   </si>
   <si>
-    <t>August</t>
+    <t>September</t>
   </si>
   <si>
     <t>Working days per month</t>
@@ -424,7 +488,7 @@
     <t>days/month</t>
   </si>
   <si>
-    <t>September</t>
+    <t>October</t>
   </si>
   <si>
     <t>Regular labor cost per worker per month</t>
@@ -436,7 +500,7 @@
     <t>$/worker/month</t>
   </si>
   <si>
-    <t>October</t>
+    <t>November</t>
   </si>
   <si>
     <t>Cost to hire one worker</t>
@@ -448,7 +512,7 @@
     <t>$/worker</t>
   </si>
   <si>
-    <t>November</t>
+    <t>December</t>
   </si>
   <si>
     <t>Cost to lay off one worker</t>
@@ -457,9 +521,6 @@
     <t>LayoffCost</t>
   </si>
   <si>
-    <t>December</t>
-  </si>
-  <si>
     <t>Cost to hold one bottle for one month</t>
   </si>
   <si>
@@ -508,6 +569,9 @@
     <t>bottles/month</t>
   </si>
   <si>
+    <t>Planning policies — how your company handles safety stock, backorders and workers</t>
+  </si>
+  <si>
     <t>Demand</t>
   </si>
   <si>
@@ -898,7 +962,7 @@
     <t>model_version</t>
   </si>
   <si>
-    <t>5.0.0</t>
+    <t>5.1.0</t>
   </si>
   <si>
     <t>seed</t>
@@ -907,7 +971,7 @@
     <t>config_hash</t>
   </si>
   <si>
-    <t>fdf36332bcdfa8fc</t>
+    <t>b2308c1b38e5432c</t>
   </si>
   <si>
     <t>student_id</t>
@@ -922,13 +986,13 @@
     <t>created_utc</t>
   </si>
   <si>
-    <t>2026-10-19T18:53:50Z</t>
+    <t>2026-10-19T19:43:03Z</t>
   </si>
   <si>
     <t>workbook_id</t>
   </si>
   <si>
-    <t>37f0fdb5e0a0</t>
+    <t>2d7ec47b698f</t>
   </si>
 </sst>
 </file>
@@ -1066,7 +1130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1139,6 +1203,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1449,7 +1514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:D41"/>
+  <dimension ref="B1:D59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -1501,7 +1566,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="7" t="s">
         <v>9</v>
       </c>
@@ -1510,7 +1575,7 @@
       </c>
       <c r="D9" s="37"/>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
         <v>11</v>
       </c>
@@ -1519,7 +1584,7 @@
       </c>
       <c r="D10" s="37"/>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="7" t="s">
         <v>13</v>
       </c>
@@ -1528,7 +1593,7 @@
       </c>
       <c r="D11" s="37"/>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
         <v>15</v>
       </c>
@@ -1537,7 +1602,7 @@
       </c>
       <c r="D12" s="37"/>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="7" t="s">
         <v>17</v>
       </c>
@@ -1580,149 +1645,262 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="2:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="38" t="s">
+    <row r="22" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="37"/>
+      <c r="C22" s="38" t="s">
+        <v>26</v>
+      </c>
       <c r="D22" s="37"/>
     </row>
-    <row r="24" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B24" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B25" s="13" t="s">
+    <row r="23" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C23" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D23" s="37"/>
+    </row>
+    <row r="24" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C24" s="38" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B26" s="13" t="s">
+      <c r="D24" s="37"/>
+    </row>
+    <row r="25" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D25" s="37"/>
+    </row>
+    <row r="26" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="38" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B27" s="13" t="s">
+      <c r="D26" s="37"/>
+    </row>
+    <row r="28" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C28" s="38" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B28" s="13" t="s">
+      <c r="D28" s="37"/>
+    </row>
+    <row r="29" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C29" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D29" s="37"/>
+    </row>
+    <row r="30" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C30" s="38" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B29" s="13" t="s">
+      <c r="D30" s="37"/>
+    </row>
+    <row r="31" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C31" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D31" s="37"/>
+    </row>
+    <row r="32" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C32" s="38" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B30" s="13" t="s">
+      <c r="D32" s="37"/>
+    </row>
+    <row r="33" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C33" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D33" s="37"/>
+    </row>
+    <row r="35" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="7" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B31" s="13" t="s">
+      <c r="C35" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D35" s="37"/>
+    </row>
+    <row r="36" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C36" s="38" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="13" t="s">
+      <c r="D36" s="37"/>
+    </row>
+    <row r="37" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C37" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D37" s="37"/>
+    </row>
+    <row r="38" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C38" s="38" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" s="13" t="s">
+      <c r="D38" s="37"/>
+    </row>
+    <row r="39" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C39" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D39" s="37"/>
+    </row>
+    <row r="42" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B42" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="13" t="s">
+    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B43" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C43" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B35" s="13" t="s">
+    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B44" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C44" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B36" s="13" t="s">
+    <row r="45" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B45" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C45" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B37" s="13" t="s">
+    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B46" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C46" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B38" s="13" t="s">
+    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B47" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C47" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B40" s="2" t="s">
+    <row r="48" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B48" s="13" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B41" s="2" t="s">
+      <c r="C48" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B49" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C49" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B50" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C50" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B51" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C51" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B52" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C52" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B53" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C53" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B54" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C54" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B55" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C55" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B56" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C56" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B58" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B59" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
-  <mergeCells count="7">
+  <mergeCells count="22">
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C13:D13"/>
     <mergeCell ref="D4:D6"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C26:D26"/>
     <mergeCell ref="C9:D9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1731,7 +1909,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1745,354 +1923,622 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="B6" s="15">
         <v>7000</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="F6" s="15">
         <v>2400</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="B7" s="15">
         <v>6000</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="F7" s="15">
-        <v>2400</v>
+        <v>0</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B8" s="15">
         <v>7000</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="F8" s="15">
-        <v>0</v>
+        <v>2400</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="B9" s="15">
         <v>11500</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="F9" s="15">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="B10" s="15">
         <v>13000</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="F10" s="15">
-        <v>8</v>
+        <v>30000</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="B11" s="15">
         <v>16500</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="F11" s="15">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="B12" s="15">
         <v>18500</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="F12" s="15">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="B13" s="15">
         <v>14000</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="F13" s="15">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="B14" s="15">
         <v>10500</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="F14" s="18">
-        <v>3200</v>
+        <v>114</v>
+      </c>
+      <c r="F14" s="15">
+        <v>25</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B15" s="15">
         <v>9000</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="F15" s="18">
-        <v>600</v>
+        <v>3200</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="H15" s="16" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="B16" s="15">
         <v>7000</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="F16" s="18">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="H16" s="16" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="B17" s="15">
         <v>6000</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="F17" s="18">
-        <v>0.25</v>
+        <v>900</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="H17" s="16" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E18" s="16" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="F18" s="18">
-        <v>1.5</v>
+        <v>0.25</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E19" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="F19" s="19">
-        <v>0.2</v>
+        <v>131</v>
+      </c>
+      <c r="F19" s="18">
+        <v>1.5</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="H19" s="16" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E20" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="F20" s="18">
-        <v>4.5</v>
+        <v>133</v>
+      </c>
+      <c r="F20" s="19">
+        <v>0.2</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E21" s="16" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="F21" s="18">
-        <v>5.25</v>
+        <v>4.5</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E22" s="16" t="s">
-        <v>121</v>
-      </c>
-      <c r="F22" s="15">
+        <v>139</v>
+      </c>
+      <c r="F22" s="18">
+        <v>5.25</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="H22" s="16" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E23" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="F23" s="15">
         <v>5000</v>
       </c>
-      <c r="G22" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="H22" s="16" t="s">
-        <v>123</v>
-      </c>
+      <c r="G23" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="H23" s="16" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="37"/>
+    </row>
+    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="38" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="37"/>
+    </row>
+    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="37"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="37"/>
+      <c r="E29" s="37"/>
+      <c r="F29" s="37"/>
+      <c r="G29" s="37"/>
+      <c r="H29" s="37"/>
+    </row>
+    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="38" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="37"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="37"/>
+      <c r="E30" s="37"/>
+      <c r="F30" s="37"/>
+      <c r="G30" s="37"/>
+      <c r="H30" s="37"/>
+    </row>
+    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="37"/>
+      <c r="H31" s="37"/>
+    </row>
+    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" s="37"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="37"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="37"/>
+      <c r="F34" s="37"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="37"/>
+    </row>
+    <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="37"/>
+    </row>
+    <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="38" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="37"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="37"/>
+      <c r="E36" s="37"/>
+      <c r="F36" s="37"/>
+      <c r="G36" s="37"/>
+      <c r="H36" s="37"/>
+    </row>
+    <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B37" s="37"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="37"/>
+      <c r="E37" s="37"/>
+      <c r="F37" s="37"/>
+      <c r="G37" s="37"/>
+      <c r="H37" s="37"/>
+    </row>
+    <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="B38" s="37"/>
+      <c r="C38" s="37"/>
+      <c r="D38" s="37"/>
+      <c r="E38" s="37"/>
+      <c r="F38" s="37"/>
+      <c r="G38" s="37"/>
+      <c r="H38" s="37"/>
+    </row>
+    <row r="39" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="B39" s="37"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="37"/>
+      <c r="E39" s="37"/>
+      <c r="F39" s="37"/>
+      <c r="G39" s="37"/>
+      <c r="H39" s="37"/>
+    </row>
+    <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B40" s="37"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="37"/>
+      <c r="E40" s="37"/>
+      <c r="F40" s="37"/>
+      <c r="G40" s="37"/>
+      <c r="H40" s="37"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B42" s="37"/>
+      <c r="C42" s="37"/>
+      <c r="D42" s="37"/>
+      <c r="E42" s="37"/>
+      <c r="F42" s="37"/>
+      <c r="G42" s="37"/>
+      <c r="H42" s="37"/>
+    </row>
+    <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="38" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" s="37"/>
+      <c r="C43" s="37"/>
+      <c r="D43" s="37"/>
+      <c r="E43" s="37"/>
+      <c r="F43" s="37"/>
+      <c r="G43" s="37"/>
+      <c r="H43" s="37"/>
+    </row>
+    <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="B44" s="37"/>
+      <c r="C44" s="37"/>
+      <c r="D44" s="37"/>
+      <c r="E44" s="37"/>
+      <c r="F44" s="37"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="37"/>
+    </row>
+    <row r="45" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="B45" s="37"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+      <c r="E45" s="37"/>
+      <c r="F45" s="37"/>
+      <c r="G45" s="37"/>
+      <c r="H45" s="37"/>
+    </row>
+    <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="B46" s="37"/>
+      <c r="C46" s="37"/>
+      <c r="D46" s="37"/>
+      <c r="E46" s="37"/>
+      <c r="F46" s="37"/>
+      <c r="G46" s="37"/>
+      <c r="H46" s="37"/>
+    </row>
+    <row r="47" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="B47" s="37"/>
+      <c r="C47" s="37"/>
+      <c r="D47" s="37"/>
+      <c r="E47" s="37"/>
+      <c r="F47" s="37"/>
+      <c r="G47" s="37"/>
+      <c r="H47" s="37"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
+  <mergeCells count="19">
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A37:H37"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2108,52 +2554,52 @@
   <sheetData>
     <row r="1" spans="1:30" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="K1" s="21" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
       <c r="L1" s="21" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="M1" s="21" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="N1" s="21" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="O1" s="21" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="P1" s="21" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="Q1" s="21"/>
       <c r="R1" s="21"/>
@@ -2172,7 +2618,7 @@
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="B2" s="15">
         <v>7000</v>
@@ -2182,7 +2628,7 @@
         <v>2400</v>
       </c>
       <c r="D2" s="22">
-        <f>0</f>
+        <f>BeginBackorders</f>
         <v>0</v>
       </c>
       <c r="E2" s="22">
@@ -2250,7 +2696,7 @@
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="B3" s="15">
         <v>6000</v>
@@ -2328,7 +2774,7 @@
     </row>
     <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B4" s="15">
         <v>7000</v>
@@ -2406,7 +2852,7 @@
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="B5" s="15">
         <v>11500</v>
@@ -2484,7 +2930,7 @@
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="B6" s="15">
         <v>13000</v>
@@ -2562,7 +3008,7 @@
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="B7" s="15">
         <v>16500</v>
@@ -2640,7 +3086,7 @@
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="B8" s="15">
         <v>18500</v>
@@ -2718,7 +3164,7 @@
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="B9" s="15">
         <v>14000</v>
@@ -2796,7 +3242,7 @@
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="B10" s="15">
         <v>10500</v>
@@ -2874,7 +3320,7 @@
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B11" s="15">
         <v>9000</v>
@@ -2952,7 +3398,7 @@
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="B12" s="15">
         <v>7000</v>
@@ -3030,7 +3476,7 @@
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="B13" s="15">
         <v>6000</v>
@@ -3108,7 +3554,7 @@
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="23" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="B14" s="24"/>
       <c r="C14" s="25"/>
@@ -3169,24 +3615,24 @@
     </row>
     <row r="16" spans="1:30" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
-        <v>141</v>
-      </c>
-      <c r="B17" s="40"/>
+      <c r="A17" s="40" t="s">
+        <v>162</v>
+      </c>
+      <c r="B17" s="41"/>
       <c r="C17" s="22">
         <f>BottlesPerHour*HoursPerDay*DaysPerMonth</f>
         <v>1000</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="39" t="s">
-        <v>142</v>
-      </c>
-      <c r="B18" s="40"/>
+      <c r="A18" s="40" t="s">
+        <v>163</v>
+      </c>
+      <c r="B18" s="41"/>
       <c r="C18" s="22">
         <f>EndTarget</f>
         <v>0</v>
@@ -3194,12 +3640,12 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -3224,52 +3670,52 @@
   <sheetData>
     <row r="1" spans="1:30" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="K1" s="21" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
       <c r="L1" s="21" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="M1" s="21" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="N1" s="21" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="O1" s="21" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="P1" s="21" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="Q1" s="21"/>
       <c r="R1" s="21"/>
@@ -3288,7 +3734,7 @@
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="B2" s="15">
         <v>7000</v>
@@ -3298,7 +3744,7 @@
         <v>2400</v>
       </c>
       <c r="D2" s="22">
-        <f>0</f>
+        <f>BeginBackorders</f>
         <v>0</v>
       </c>
       <c r="E2" s="22">
@@ -3366,7 +3812,7 @@
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="B3" s="15">
         <v>6000</v>
@@ -3444,7 +3890,7 @@
     </row>
     <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B4" s="15">
         <v>7000</v>
@@ -3522,7 +3968,7 @@
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="B5" s="15">
         <v>11500</v>
@@ -3600,7 +4046,7 @@
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="B6" s="15">
         <v>13000</v>
@@ -3678,7 +4124,7 @@
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="B7" s="15">
         <v>16500</v>
@@ -3756,7 +4202,7 @@
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="B8" s="15">
         <v>18500</v>
@@ -3834,7 +4280,7 @@
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="B9" s="15">
         <v>14000</v>
@@ -3912,7 +4358,7 @@
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="B10" s="15">
         <v>10500</v>
@@ -3990,7 +4436,7 @@
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B11" s="15">
         <v>9000</v>
@@ -4068,7 +4514,7 @@
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="B12" s="15">
         <v>7000</v>
@@ -4146,7 +4592,7 @@
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="B13" s="15">
         <v>6000</v>
@@ -4224,7 +4670,7 @@
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="23" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="B14" s="24"/>
       <c r="C14" s="25"/>
@@ -4285,54 +4731,54 @@
     </row>
     <row r="16" spans="1:30" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
-        <v>141</v>
-      </c>
-      <c r="B17" s="40"/>
+      <c r="A17" s="40" t="s">
+        <v>162</v>
+      </c>
+      <c r="B17" s="41"/>
       <c r="C17" s="22">
         <f>BottlesPerHour*HoursPerDay*DaysPerMonth</f>
         <v>1000</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="39" t="s">
-        <v>145</v>
-      </c>
-      <c r="B18" s="40"/>
+      <c r="A18" s="40" t="s">
+        <v>166</v>
+      </c>
+      <c r="B18" s="41"/>
       <c r="C18" s="22">
         <f>EndTarget</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="39" t="s">
-        <v>146</v>
-      </c>
-      <c r="B19" s="40"/>
+      <c r="A19" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="B19" s="41"/>
       <c r="C19" s="22">
         <f>SUM(B2:B13)</f>
         <v>126000</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="39" t="s">
-        <v>147</v>
-      </c>
-      <c r="B20" s="40"/>
+      <c r="A20" s="40" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20" s="41"/>
       <c r="C20" s="22">
-        <f>(C19+C18-BeginInv)/12</f>
+        <f>(C19+C18-BeginInv+BeginBackorders)/12</f>
         <v>10300</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="39" t="s">
-        <v>148</v>
-      </c>
-      <c r="B21" s="40"/>
+      <c r="A21" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="B21" s="41"/>
       <c r="C21" s="22">
         <f>ROUNDUP(C20/C17,0)</f>
         <v>11</v>
@@ -4340,12 +4786,12 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -4373,70 +4819,70 @@
   <sheetData>
     <row r="1" spans="1:30" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="F1" s="21" t="s">
+        <v>171</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="H1" s="21" t="s">
+        <v>173</v>
+      </c>
+      <c r="I1" s="21" t="s">
+        <v>174</v>
+      </c>
+      <c r="J1" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="K1" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="L1" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="M1" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="N1" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="O1" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="K1" s="21" t="s">
-        <v>129</v>
-      </c>
-      <c r="L1" s="21" t="s">
-        <v>130</v>
-      </c>
-      <c r="M1" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="N1" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="O1" s="21" t="s">
-        <v>133</v>
-      </c>
       <c r="P1" s="21" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="Q1" s="21" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="R1" s="21" t="s">
-        <v>155</v>
+        <v>176</v>
       </c>
       <c r="S1" s="21" t="s">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="T1" s="21" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="U1" s="21" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="V1" s="21" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="W1" s="21"/>
       <c r="X1" s="21"/>
@@ -4449,7 +4895,7 @@
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="B2" s="15">
         <v>7000</v>
@@ -4459,7 +4905,7 @@
         <v>2400</v>
       </c>
       <c r="D2" s="22">
-        <f>0</f>
+        <f>BeginBackorders</f>
         <v>0</v>
       </c>
       <c r="E2" s="22">
@@ -4541,7 +4987,7 @@
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="B3" s="15">
         <v>6000</v>
@@ -4633,7 +5079,7 @@
     </row>
     <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B4" s="15">
         <v>7000</v>
@@ -4725,7 +5171,7 @@
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="B5" s="15">
         <v>11500</v>
@@ -4817,7 +5263,7 @@
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="B6" s="15">
         <v>13000</v>
@@ -4909,7 +5355,7 @@
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="B7" s="15">
         <v>16500</v>
@@ -5001,7 +5447,7 @@
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="B8" s="15">
         <v>18500</v>
@@ -5093,7 +5539,7 @@
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="B9" s="15">
         <v>14000</v>
@@ -5185,7 +5631,7 @@
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="B10" s="15">
         <v>10500</v>
@@ -5277,7 +5723,7 @@
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B11" s="15">
         <v>9000</v>
@@ -5369,7 +5815,7 @@
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="B12" s="15">
         <v>7000</v>
@@ -5461,7 +5907,7 @@
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="B13" s="15">
         <v>6000</v>
@@ -5553,7 +5999,7 @@
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="23" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="B14" s="24"/>
       <c r="C14" s="25"/>
@@ -5632,24 +6078,24 @@
     </row>
     <row r="16" spans="1:30" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
-        <v>141</v>
-      </c>
-      <c r="B17" s="40"/>
+      <c r="A17" s="40" t="s">
+        <v>162</v>
+      </c>
+      <c r="B17" s="41"/>
       <c r="C17" s="22">
         <f>BottlesPerHour*HoursPerDay*DaysPerMonth</f>
         <v>1000</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="39" t="s">
-        <v>157</v>
-      </c>
-      <c r="B18" s="40"/>
+      <c r="A18" s="40" t="s">
+        <v>178</v>
+      </c>
+      <c r="B18" s="41"/>
       <c r="C18" s="22">
         <f>C17*OTLimitPct</f>
         <v>200</v>
@@ -5657,17 +6103,17 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>159</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -5693,29 +6139,29 @@
   <sheetData>
     <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>164</v>
+        <v>185</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>165</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
       <c r="B4" s="26">
         <f>'Chase Plan'!K14</f>
@@ -5730,12 +6176,12 @@
         <v>422400</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>168</v>
+        <v>189</v>
       </c>
       <c r="B5" s="26">
         <f>'Chase Plan'!L14</f>
@@ -5750,12 +6196,12 @@
         <v>1800</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="B6" s="26">
         <f>'Chase Plan'!M14</f>
@@ -5770,48 +6216,48 @@
         <v>0</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
-        <v>170</v>
+        <v>191</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>171</v>
+        <v>192</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>171</v>
+        <v>192</v>
       </c>
       <c r="D7" s="26">
         <f>'Hybrid Plan'!R14</f>
         <v>13500</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>172</v>
+        <v>193</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>171</v>
+        <v>192</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>171</v>
+        <v>192</v>
       </c>
       <c r="D8" s="26">
         <f>'Hybrid Plan'!S14</f>
         <v>0</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>172</v>
+        <v>193</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>174</v>
+        <v>195</v>
       </c>
       <c r="B9" s="26">
         <f>'Chase Plan'!N14</f>
@@ -5826,12 +6272,12 @@
         <v>23225</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
-        <v>175</v>
+        <v>196</v>
       </c>
       <c r="B10" s="26">
         <f>'Chase Plan'!O14</f>
@@ -5846,12 +6292,12 @@
         <v>150</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="28" t="s">
-        <v>176</v>
+        <v>197</v>
       </c>
       <c r="B11" s="29">
         <f>'Chase Plan'!P14</f>
@@ -5866,12 +6312,12 @@
         <v>461075</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="B12" s="30">
         <f>'Chase Plan'!G14</f>
@@ -5886,12 +6332,12 @@
         <v>3</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
-        <v>179</v>
+        <v>200</v>
       </c>
       <c r="B13" s="30">
         <f>'Chase Plan'!H14</f>
@@ -5906,12 +6352,12 @@
         <v>0</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="B14" s="30">
         <f>MAX('Chase Plan'!F2:F13)</f>
@@ -5926,12 +6372,12 @@
         <v>11</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>181</v>
+        <v>202</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
-        <v>182</v>
+        <v>203</v>
       </c>
       <c r="B15" s="30">
         <f>MAX('Chase Plan'!I2:I13)</f>
@@ -5946,12 +6392,12 @@
         <v>15400</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>181</v>
+        <v>202</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
-        <v>183</v>
+        <v>204</v>
       </c>
       <c r="B16" s="30">
         <f>COUNTIF('Chase Plan'!J2:J13,"&gt;0")</f>
@@ -5966,50 +6412,50 @@
         <v>1</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>184</v>
+        <v>205</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="28" t="s">
-        <v>185</v>
+        <v>206</v>
       </c>
       <c r="B18" s="31" t="str">
         <f>IF(B11&lt;C11,"Chase","Level")</f>
         <v>Chase</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="28" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
       <c r="B19" s="26">
         <f>ABS(B11-C11)</f>
         <v>63375</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="28" t="s">
-        <v>189</v>
+        <v>210</v>
       </c>
       <c r="B21" s="31" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="32" t="s">
-        <v>191</v>
-      </c>
-      <c r="B22" s="41" t="s">
-        <v>192</v>
+        <v>212</v>
+      </c>
+      <c r="B22" s="42" t="s">
+        <v>213</v>
       </c>
       <c r="C22" s="37"/>
       <c r="D22" s="37"/>
@@ -6017,7 +6463,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="36" t="s">
-        <v>193</v>
+        <v>214</v>
       </c>
       <c r="B23" s="37"/>
       <c r="C23" s="37"/>
@@ -6096,215 +6542,215 @@
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>194</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>196</v>
+        <v>217</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>197</v>
+        <v>218</v>
       </c>
       <c r="C4" s="37"/>
     </row>
     <row r="5" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="C5" s="37"/>
     </row>
     <row r="6" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>201</v>
+        <v>222</v>
       </c>
       <c r="C6" s="37"/>
     </row>
     <row r="7" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>202</v>
+        <v>223</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
       <c r="C7" s="37"/>
     </row>
     <row r="8" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>204</v>
+        <v>225</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>205</v>
+        <v>226</v>
       </c>
       <c r="C8" s="37"/>
     </row>
     <row r="9" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>206</v>
+        <v>227</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>207</v>
+        <v>228</v>
       </c>
       <c r="C9" s="37"/>
     </row>
     <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>208</v>
+        <v>229</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>209</v>
+        <v>230</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>212</v>
+        <v>233</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>213</v>
+        <v>234</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>214</v>
+        <v>235</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>215</v>
+        <v>236</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>216</v>
+        <v>237</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>220</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>221</v>
+        <v>242</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>222</v>
+        <v>243</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>223</v>
+        <v>244</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>224</v>
+        <v>245</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>225</v>
+        <v>246</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>226</v>
+        <v>247</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>227</v>
+        <v>248</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>228</v>
+        <v>249</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>229</v>
+        <v>250</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>230</v>
+        <v>251</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>231</v>
+        <v>252</v>
       </c>
       <c r="B21" s="38" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="C21" s="37"/>
     </row>
     <row r="22" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>233</v>
+        <v>254</v>
       </c>
       <c r="B22" s="38" t="s">
-        <v>234</v>
+        <v>255</v>
       </c>
       <c r="C22" s="37"/>
     </row>
     <row r="23" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>235</v>
+        <v>256</v>
       </c>
       <c r="B23" s="38" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
       <c r="C23" s="37"/>
     </row>
     <row r="24" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>237</v>
+        <v>258</v>
       </c>
       <c r="B24" s="38" t="s">
-        <v>238</v>
+        <v>259</v>
       </c>
       <c r="C24" s="37"/>
     </row>
     <row r="25" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>239</v>
+        <v>260</v>
       </c>
       <c r="B25" s="38" t="s">
-        <v>240</v>
+        <v>261</v>
       </c>
       <c r="C25" s="37"/>
     </row>
     <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>241</v>
+        <v>262</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>242</v>
+        <v>263</v>
       </c>
       <c r="B28" s="37"/>
       <c r="C28" s="37"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>243</v>
+        <v>264</v>
       </c>
       <c r="B30" s="34">
         <v>0.25</v>
@@ -6312,7 +6758,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>244</v>
+        <v>265</v>
       </c>
       <c r="B31" s="35">
         <v>1200</v>
@@ -6321,7 +6767,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>245</v>
+        <v>266</v>
       </c>
       <c r="B32" s="35">
         <v>850</v>
@@ -6330,7 +6776,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>246</v>
+        <v>267</v>
       </c>
       <c r="B33" s="35">
         <v>1500</v>
@@ -6339,7 +6785,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>247</v>
+        <v>268</v>
       </c>
       <c r="B34" s="35">
         <v>2300</v>
@@ -6348,7 +6794,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>248</v>
+        <v>269</v>
       </c>
       <c r="B35" s="35">
         <v>975</v>
@@ -6357,7 +6803,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>249</v>
+        <v>270</v>
       </c>
       <c r="B36" s="35">
         <v>1840</v>
@@ -6391,15 +6837,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>250</v>
+        <v>271</v>
       </c>
       <c r="B1" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>252</v>
+        <v>273</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -6407,15 +6853,15 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>253</v>
+        <v>274</v>
       </c>
       <c r="B3" t="s">
-        <v>254</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>255</v>
+        <v>276</v>
       </c>
       <c r="B4">
         <v>7</v>
@@ -6423,15 +6869,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="B5" t="s">
-        <v>257</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>258</v>
+        <v>279</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
@@ -6439,7 +6885,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>259</v>
+        <v>280</v>
       </c>
       <c r="B7" t="s">
         <v>3</v>
@@ -6447,23 +6893,23 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>261</v>
+        <v>282</v>
       </c>
       <c r="B9" t="s">
-        <v>262</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>263</v>
+        <v>284</v>
       </c>
       <c r="B10" t="s">
-        <v>264</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>